<commit_message>
Changed mapping and categories
</commit_message>
<xml_diff>
--- a/gsbpm/apps/systemer/koblinger.xlsx
+++ b/gsbpm/apps/systemer/koblinger.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10525"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ssbno-my.sharepoint.com/personal/thb_ssb_no/Documents/Documents/GitHub/dataviz-resources/gsbpm/apps/systemer/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/obv/Projects/github/diverse/thomasbjornskau/dataviz-resources/gsbpm/apps/systemer/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="11_A954B997964A36FEE87DD0355E10363B1A80FAC5" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3182C1F3-64E2-4476-854F-7678118DDEB7}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25BEE3A1-0995-FD4B-ADFA-C255736EA7EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="43560" yWindow="5520" windowWidth="24960" windowHeight="17000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Koblinger" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="31">
   <si>
     <t>SYSTEMNAVN</t>
   </si>
@@ -37,45 +37,21 @@
     <t>Kudoc</t>
   </si>
   <si>
-    <t>2.2</t>
-  </si>
-  <si>
     <t>Helt</t>
   </si>
   <si>
-    <t>Noe tekst her</t>
-  </si>
-  <si>
-    <t>3.1</t>
-  </si>
-  <si>
     <t>Delvis</t>
   </si>
   <si>
-    <t>RespReg</t>
-  </si>
-  <si>
-    <t>4.1</t>
-  </si>
-  <si>
     <t>Amor</t>
   </si>
   <si>
-    <t>5.1</t>
-  </si>
-  <si>
     <t>A3Admin</t>
   </si>
   <si>
-    <t>5.2</t>
-  </si>
-  <si>
     <t>DaplaLab</t>
   </si>
   <si>
-    <t>6.2</t>
-  </si>
-  <si>
     <t>Vardef</t>
   </si>
   <si>
@@ -85,20 +61,65 @@
     <t>Klass</t>
   </si>
   <si>
-    <t>Statreg</t>
-  </si>
-  <si>
-    <t>6.3</t>
-  </si>
-  <si>
-    <t>1.2</t>
+    <t>Delomat</t>
+  </si>
+  <si>
+    <t>DaplaCtrl</t>
+  </si>
+  <si>
+    <t>Webscraping og enkle API</t>
+  </si>
+  <si>
+    <t>DataCollector</t>
+  </si>
+  <si>
+    <t>API-innhenting</t>
+  </si>
+  <si>
+    <t>Datakatalog</t>
+  </si>
+  <si>
+    <t>Sjekke om data allerede finnes internt</t>
+  </si>
+  <si>
+    <t>Editeringsrammeverk</t>
+  </si>
+  <si>
+    <t>Kildomat</t>
+  </si>
+  <si>
+    <t>Kodeverk og klassifikasjoner</t>
+  </si>
+  <si>
+    <t>Metadata om innsamlinger</t>
+  </si>
+  <si>
+    <t>Benytter informasjon fra Kudoc</t>
+  </si>
+  <si>
+    <t>Metodebibliotek</t>
+  </si>
+  <si>
+    <t>Respondentregister</t>
+  </si>
+  <si>
+    <t>Statistikkregisteret</t>
+  </si>
+  <si>
+    <t>Metadata om statistikkproduker og publisering</t>
+  </si>
+  <si>
+    <t>Sjekke om variabler allerede er definert internt</t>
+  </si>
+  <si>
+    <t>Variabeldefinisjoner</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -110,6 +131,14 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -135,7 +164,7 @@
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -438,16 +467,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D12"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:D41"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="1" max="1" width="18.33203125" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
     <col min="4" max="4" width="50" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -461,161 +490,480 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2" t="s">
-        <v>5</v>
+        <v>18</v>
+      </c>
+      <c r="B2">
+        <v>1.5</v>
       </c>
       <c r="C2" t="s">
         <v>6</v>
       </c>
       <c r="D2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" t="s">
-        <v>8</v>
+        <v>10</v>
+      </c>
+      <c r="B3">
+        <v>1.5</v>
       </c>
       <c r="C3" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="D3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" t="s">
-        <v>11</v>
+        <v>27</v>
+      </c>
+      <c r="B4">
+        <v>2.1</v>
       </c>
       <c r="C4" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="D4" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>12</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="C5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D5" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="C6" t="s">
+        <v>5</v>
+      </c>
+      <c r="D6" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="C7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D7" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>4</v>
+      </c>
+      <c r="B8">
+        <v>2.4</v>
+      </c>
+      <c r="C8" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9">
+        <v>3.1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>5</v>
+      </c>
+      <c r="D9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>16</v>
+      </c>
+      <c r="B10">
+        <v>3.1</v>
+      </c>
+      <c r="C10" t="s">
+        <v>5</v>
+      </c>
+      <c r="D10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>4</v>
+      </c>
+      <c r="B11">
+        <v>3.1</v>
+      </c>
+      <c r="C11" t="s">
+        <v>6</v>
+      </c>
+      <c r="D11" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>9</v>
+      </c>
+      <c r="B12">
+        <v>3.5</v>
+      </c>
+      <c r="C12" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>9</v>
+      </c>
+      <c r="B13">
+        <v>3.6</v>
+      </c>
+      <c r="C13" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>9</v>
+      </c>
+      <c r="B14">
+        <v>3.7</v>
+      </c>
+      <c r="C14" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>4</v>
+      </c>
+      <c r="B15">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="C15" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A16" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B16" s="2">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>26</v>
+      </c>
+      <c r="B17">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="C17" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>8</v>
+      </c>
+      <c r="B18">
+        <v>4.2</v>
+      </c>
+      <c r="C18" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>7</v>
+      </c>
+      <c r="B19">
+        <v>4.2</v>
+      </c>
+      <c r="C19" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>26</v>
+      </c>
+      <c r="B20">
+        <v>4.2</v>
+      </c>
+      <c r="C20" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>8</v>
+      </c>
+      <c r="B21">
+        <v>4.3</v>
+      </c>
+      <c r="C21" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>7</v>
+      </c>
+      <c r="B22">
+        <v>4.3</v>
+      </c>
+      <c r="C22" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>16</v>
+      </c>
+      <c r="B23">
+        <v>4.3</v>
+      </c>
+      <c r="C23" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>26</v>
+      </c>
+      <c r="B24">
+        <v>4.3</v>
+      </c>
+      <c r="C24" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>8</v>
+      </c>
+      <c r="B25">
+        <v>4.4000000000000004</v>
+      </c>
+      <c r="C25" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>7</v>
+      </c>
+      <c r="B26">
+        <v>4.4000000000000004</v>
+      </c>
+      <c r="C26" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A27" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B27" s="2">
+        <v>4.4000000000000004</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D27" s="2"/>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A28" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B28" s="2">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D28" s="2"/>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A29" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>14</v>
-      </c>
-      <c r="B6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C6" t="s">
-        <v>9</v>
-      </c>
-      <c r="D6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>16</v>
-      </c>
-      <c r="B7" t="s">
-        <v>17</v>
-      </c>
-      <c r="C7" t="s">
-        <v>9</v>
-      </c>
-      <c r="D7" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>18</v>
-      </c>
-      <c r="B8" t="s">
-        <v>17</v>
-      </c>
-      <c r="C8" t="s">
-        <v>9</v>
-      </c>
-      <c r="D8" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>19</v>
-      </c>
-      <c r="B9" t="s">
-        <v>17</v>
-      </c>
-      <c r="C9" t="s">
-        <v>9</v>
-      </c>
-      <c r="D9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+      <c r="B29" s="2">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D29" s="2"/>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>12</v>
+      </c>
+      <c r="B30">
+        <v>5.2</v>
+      </c>
+      <c r="C30" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A31" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B10" t="s">
-        <v>17</v>
-      </c>
-      <c r="C10" t="s">
-        <v>9</v>
-      </c>
-      <c r="D10" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>21</v>
-      </c>
-      <c r="B11" t="s">
-        <v>22</v>
-      </c>
-      <c r="C11" t="s">
-        <v>9</v>
-      </c>
-      <c r="D11" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>21</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C12" t="s">
-        <v>6</v>
-      </c>
-      <c r="D12" t="s">
-        <v>7</v>
+      <c r="B31" s="2">
+        <v>5.4</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
+        <v>11</v>
+      </c>
+      <c r="B32">
+        <v>5.8</v>
+      </c>
+      <c r="C32" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
+        <v>10</v>
+      </c>
+      <c r="B33">
+        <v>5.8</v>
+      </c>
+      <c r="C33" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>9</v>
+      </c>
+      <c r="B34">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="C34" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
+        <v>9</v>
+      </c>
+      <c r="B35">
+        <v>5.2</v>
+      </c>
+      <c r="C35" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
+        <v>9</v>
+      </c>
+      <c r="B36">
+        <v>5.3</v>
+      </c>
+      <c r="C36" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
+        <v>9</v>
+      </c>
+      <c r="B37">
+        <v>5.4</v>
+      </c>
+      <c r="C37" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
+        <v>9</v>
+      </c>
+      <c r="B38">
+        <v>5.5</v>
+      </c>
+      <c r="C38" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
+        <v>9</v>
+      </c>
+      <c r="B39">
+        <v>5.6</v>
+      </c>
+      <c r="C39" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
+        <v>9</v>
+      </c>
+      <c r="B40">
+        <v>5.7</v>
+      </c>
+      <c r="C40" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
+        <v>9</v>
+      </c>
+      <c r="B41">
+        <v>5.8</v>
+      </c>
+      <c r="C41" t="s">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D33">
+    <sortCondition ref="B2:B33"/>
+  </sortState>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Mer fram og tilbake
</commit_message>
<xml_diff>
--- a/gsbpm/apps/systemer/koblinger.xlsx
+++ b/gsbpm/apps/systemer/koblinger.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/obv/Projects/github/diverse/thomasbjornskau/dataviz-resources/gsbpm/apps/systemer/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2EDCE63-5450-4A4A-B7CA-6F2EFBB4A869}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{940011E2-3C84-9D42-945A-C49DE914A76E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="43560" yWindow="5520" windowWidth="24960" windowHeight="17000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="35260" yWindow="7220" windowWidth="24960" windowHeight="17000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Koblinger" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="42">
   <si>
     <t>SYSTEMNAVN</t>
   </si>
@@ -64,15 +64,9 @@
     <t>DaplaCtrl</t>
   </si>
   <si>
-    <t>Webscraping og enkle API</t>
-  </si>
-  <si>
     <t>DataCollector</t>
   </si>
   <si>
-    <t>Datakatalog</t>
-  </si>
-  <si>
     <t>Sjekke om data allerede finnes internt</t>
   </si>
   <si>
@@ -106,18 +100,6 @@
     <t>Statistikkregister</t>
   </si>
   <si>
-    <t>Komplekse API</t>
-  </si>
-  <si>
-    <t>Personundersøkelser med intervju</t>
-  </si>
-  <si>
-    <t>Næringsundersøkelser via Altinn</t>
-  </si>
-  <si>
-    <t>Egen kode i DaplaLab</t>
-  </si>
-  <si>
     <t>Kan forberede for enkle API-er og Webscraping</t>
   </si>
   <si>
@@ -125,6 +107,45 @@
   </si>
   <si>
     <t>ssb.no</t>
+  </si>
+  <si>
+    <t>Div fellesbibliotek</t>
+  </si>
+  <si>
+    <t>Kan overføre til statistikkbank med dapla-statbank-klient</t>
+  </si>
+  <si>
+    <t>Kan tilrettelegge prefilldata til altinn med dapla-suv-tools</t>
+  </si>
+  <si>
+    <t>Tilrettelegging for personundersøkelser med intervju</t>
+  </si>
+  <si>
+    <t>Tilrettelegging for næringsundersøkelser via Altinn</t>
+  </si>
+  <si>
+    <t>U-en i Kudoc står for Utvalgsdokumentasjon</t>
+  </si>
+  <si>
+    <t>Kan kode egne løp</t>
+  </si>
+  <si>
+    <t>Metodebiblioteket har funksjoner for imputering</t>
+  </si>
+  <si>
+    <t>Metodebiblioteket har funksjoner for undertrykking og støylegging</t>
+  </si>
+  <si>
+    <t>Dataportal</t>
+  </si>
+  <si>
+    <t>Enonic CMS</t>
+  </si>
+  <si>
+    <t>DaplaLab</t>
+  </si>
+  <si>
+    <t>Kan bruke egen kode for å bygge løsning for webscraping og enkel API-innhenting</t>
   </si>
 </sst>
 </file>
@@ -479,7 +500,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D46"/>
+  <dimension ref="A1:D54"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18.33203125" customWidth="1"/>
@@ -512,9 +533,6 @@
       <c r="C2" t="s">
         <v>5</v>
       </c>
-      <c r="D2" t="s">
-        <v>30</v>
-      </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
@@ -526,6 +544,9 @@
       <c r="C3" t="s">
         <v>5</v>
       </c>
+      <c r="D3" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
@@ -559,9 +580,6 @@
       <c r="C6" t="s">
         <v>5</v>
       </c>
-      <c r="D6" t="s">
-        <v>29</v>
-      </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
@@ -573,6 +591,9 @@
       <c r="C7" t="s">
         <v>5</v>
       </c>
+      <c r="D7" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
@@ -610,7 +631,7 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>15</v>
+        <v>40</v>
       </c>
       <c r="B11">
         <v>3.1</v>
@@ -619,26 +640,29 @@
         <v>5</v>
       </c>
       <c r="D11" t="s">
-        <v>28</v>
+        <v>41</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>15</v>
+        <v>40</v>
       </c>
       <c r="B12">
-        <v>4.3</v>
+        <v>3.2</v>
       </c>
       <c r="C12" t="s">
         <v>5</v>
+      </c>
+      <c r="D12" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="B13">
-        <v>5.8</v>
+        <v>3.5</v>
       </c>
       <c r="C13" t="s">
         <v>5</v>
@@ -646,133 +670,126 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="B14">
-        <v>1.5</v>
+        <v>3.6</v>
       </c>
       <c r="C14" t="s">
-        <v>6</v>
-      </c>
-      <c r="D14" t="s">
-        <v>17</v>
+        <v>5</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A15" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B15" s="2">
-        <v>5.0999999999999996</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D15" s="2"/>
+      <c r="A15" t="s">
+        <v>40</v>
+      </c>
+      <c r="B15">
+        <v>3.7</v>
+      </c>
+      <c r="C15" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A16" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B16" s="2">
-        <v>5.4</v>
-      </c>
-      <c r="C16" s="2" t="s">
+      <c r="A16" t="s">
+        <v>40</v>
+      </c>
+      <c r="B16">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="C16" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="B17">
-        <v>3.1</v>
+        <v>4.2</v>
       </c>
       <c r="C17" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D17" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="B18">
-        <v>3.5</v>
+        <v>4.3</v>
       </c>
       <c r="C18" t="s">
-        <v>6</v>
+        <v>5</v>
+      </c>
+      <c r="D18" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="B19">
-        <v>3.6</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="C19" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="B20">
-        <v>3.7</v>
+        <v>5.2</v>
       </c>
       <c r="C20" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="B21">
-        <v>4.0999999999999996</v>
+        <v>5.3</v>
       </c>
       <c r="C21" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="B22">
-        <v>4.2</v>
+        <v>5.4</v>
       </c>
       <c r="C22" t="s">
-        <v>6</v>
-      </c>
-      <c r="D22" t="s">
-        <v>32</v>
+        <v>5</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="B23">
-        <v>4.3</v>
+        <v>5.5</v>
       </c>
       <c r="C23" t="s">
-        <v>6</v>
-      </c>
-      <c r="D23" t="s">
-        <v>33</v>
+        <v>5</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="B24">
-        <v>5.0999999999999996</v>
+        <v>5.6</v>
       </c>
       <c r="C24" t="s">
         <v>5</v>
@@ -780,10 +797,10 @@
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="B25">
-        <v>5.2</v>
+        <v>5.7</v>
       </c>
       <c r="C25" t="s">
         <v>5</v>
@@ -791,10 +808,10 @@
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="B26">
-        <v>5.3</v>
+        <v>5.8</v>
       </c>
       <c r="C26" t="s">
         <v>5</v>
@@ -802,10 +819,10 @@
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>31</v>
+        <v>14</v>
       </c>
       <c r="B27">
-        <v>5.4</v>
+        <v>3.1</v>
       </c>
       <c r="C27" t="s">
         <v>5</v>
@@ -813,10 +830,10 @@
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>31</v>
+        <v>14</v>
       </c>
       <c r="B28">
-        <v>5.5</v>
+        <v>4.3</v>
       </c>
       <c r="C28" t="s">
         <v>5</v>
@@ -824,10 +841,10 @@
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="B29">
-        <v>5.6</v>
+        <v>5.8</v>
       </c>
       <c r="C29" t="s">
         <v>5</v>
@@ -835,211 +852,318 @@
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
+        <v>38</v>
+      </c>
+      <c r="B30">
+        <v>1.5</v>
+      </c>
+      <c r="C30" t="s">
+        <v>6</v>
+      </c>
+      <c r="D30" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A31" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B31" s="2">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D31" s="2"/>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
+        <v>29</v>
+      </c>
+      <c r="B32">
+        <v>4.2</v>
+      </c>
+      <c r="C32" t="s">
+        <v>5</v>
+      </c>
+      <c r="D32" t="s">
         <v>31</v>
       </c>
-      <c r="B30">
-        <v>5.7</v>
-      </c>
-      <c r="C30" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A31" t="s">
-        <v>31</v>
-      </c>
-      <c r="B31">
-        <v>5.8</v>
-      </c>
-      <c r="C31" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A32" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="B32" s="2">
-        <v>4.4000000000000004</v>
-      </c>
-      <c r="C32" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D32" s="2"/>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="B33">
-        <v>2.2000000000000002</v>
+        <v>7.1</v>
       </c>
       <c r="C33" t="s">
         <v>5</v>
       </c>
       <c r="D33" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A34" t="s">
-        <v>11</v>
-      </c>
-      <c r="B34">
-        <v>5.2</v>
-      </c>
-      <c r="C34" t="s">
+      <c r="A34" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B34" s="2">
+        <v>5.4</v>
+      </c>
+      <c r="C34" s="2" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>4</v>
+        <v>39</v>
       </c>
       <c r="B35">
-        <v>2.2999999999999998</v>
+        <v>7.1</v>
       </c>
       <c r="C35" t="s">
         <v>5</v>
       </c>
-      <c r="D35" t="s">
-        <v>21</v>
-      </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A36" t="s">
-        <v>4</v>
-      </c>
-      <c r="B36">
-        <v>2.4</v>
-      </c>
-      <c r="C36" t="s">
-        <v>6</v>
-      </c>
+      <c r="A36" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B36" s="2">
+        <v>4.4000000000000004</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D36" s="2"/>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="B37">
-        <v>4.0999999999999996</v>
+        <v>2.2000000000000002</v>
       </c>
       <c r="C37" t="s">
-        <v>6</v>
+        <v>5</v>
+      </c>
+      <c r="D37" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A38" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B38" s="2">
-        <v>4.0999999999999996</v>
-      </c>
-      <c r="C38" s="2" t="s">
+      <c r="A38" t="s">
+        <v>11</v>
+      </c>
+      <c r="B38">
+        <v>5.2</v>
+      </c>
+      <c r="C38" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>23</v>
+        <v>4</v>
       </c>
       <c r="B39">
-        <v>4.0999999999999996</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="C39" t="s">
-        <v>6</v>
+        <v>5</v>
+      </c>
+      <c r="D39" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>23</v>
+        <v>4</v>
       </c>
       <c r="B40">
-        <v>4.2</v>
+        <v>2.4</v>
       </c>
       <c r="C40" t="s">
         <v>6</v>
       </c>
+      <c r="D40" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>23</v>
+        <v>4</v>
       </c>
       <c r="B41">
-        <v>4.3</v>
+        <v>4.0999999999999996</v>
       </c>
       <c r="C41" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A42" t="s">
-        <v>34</v>
-      </c>
-      <c r="B42">
-        <v>7.3</v>
-      </c>
-      <c r="C42" t="s">
+      <c r="A42" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B42" s="2">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="C42" s="2" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="B43">
-        <v>2.1</v>
+        <v>5.3</v>
       </c>
       <c r="C43" t="s">
         <v>5</v>
-      </c>
-      <c r="D43" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="B44">
-        <v>1.5</v>
+        <v>5.4</v>
       </c>
       <c r="C44" t="s">
         <v>5</v>
       </c>
       <c r="D44" t="s">
-        <v>25</v>
+        <v>36</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="B45">
-        <v>2.2000000000000002</v>
+        <v>5.6</v>
       </c>
       <c r="C45" t="s">
         <v>5</v>
-      </c>
-      <c r="D45" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
+        <v>20</v>
+      </c>
+      <c r="B46">
+        <v>5.7</v>
+      </c>
+      <c r="C46" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
+        <v>20</v>
+      </c>
+      <c r="B47">
+        <v>6.4</v>
+      </c>
+      <c r="C47" t="s">
+        <v>5</v>
+      </c>
+      <c r="D47" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A48" t="s">
+        <v>21</v>
+      </c>
+      <c r="B48">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="C48" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
+        <v>21</v>
+      </c>
+      <c r="B49">
+        <v>4.3</v>
+      </c>
+      <c r="C49" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A50" t="s">
+        <v>28</v>
+      </c>
+      <c r="B50">
+        <v>7.3</v>
+      </c>
+      <c r="C50" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A51" t="s">
+        <v>25</v>
+      </c>
+      <c r="B51">
+        <v>2.1</v>
+      </c>
+      <c r="C51" t="s">
+        <v>5</v>
+      </c>
+      <c r="D51" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A52" t="s">
         <v>9</v>
       </c>
-      <c r="B46">
+      <c r="B52">
+        <v>1.5</v>
+      </c>
+      <c r="C52" t="s">
+        <v>5</v>
+      </c>
+      <c r="D52" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A53" t="s">
+        <v>9</v>
+      </c>
+      <c r="B53">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="C53" t="s">
+        <v>5</v>
+      </c>
+      <c r="D53" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A54" t="s">
+        <v>9</v>
+      </c>
+      <c r="B54">
         <v>5.8</v>
       </c>
-      <c r="C46" t="s">
+      <c r="C54" t="s">
         <v>5</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D46">
-    <sortCondition ref="A2:A46"/>
-    <sortCondition ref="B2:B46"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D54">
+    <sortCondition ref="A2:A54"/>
+    <sortCondition ref="B2:B54"/>
   </sortState>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>